<commit_message>
feat: add new Excel output files for short-horizon portfolio performance analysis across weekly, monthly, and quarterly horizons for US and China markets; update Python script to enhance evaluation flexibility and data organization
</commit_message>
<xml_diff>
--- a/outputs/analysis_results/01_short-horizon portfolio performance/01_portfolio_weekly_h1_cn.xlsx
+++ b/outputs/analysis_results/01_short-horizon portfolio performance/01_portfolio_weekly_h1_cn.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,60 +447,60 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>panel: Equal-Weight</t>
+          <t>frequency</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>source sheet='equal'; Equal-weight (EW): 1/N within each decile portfolio.</t>
+          <t>weekly</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>panel: FloatCap-Weight</t>
+          <t>holding_horizon</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>source sheet='float'; Float market-cap weight at formation (CN: FloatCap / 流通市值).</t>
+          <t>R5</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>panel: TotalCap-Weight</t>
+          <t>panel: Equal-Weight</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>source sheet='total'; Total market-cap weight at formation (CN: TotalCap / 总市值).</t>
+          <t>source sheet='equal'; Equal-weight (EW): 1/N within each decile portfolio.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>panel: FloatCap-Weight</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Weekly R5 portfolio summary from step-04 CNN all_h{k}.xlsx and step-05 benchmark h{k}.xlsx.</t>
+          <t>source sheet='float'; Float market-cap weight at formation (CN: FloatCap / 流通市值).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>panel: TotalCap-Weight</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Return column: Annualized Return (raw portfolio return, annualized). NOT Annualized Active Return.</t>
+          <t>source sheet='total'; Total market-cap weight at formation (CN: TotalCap / 总市值).</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Sharpe column: Sharpe Ratio = Annualized Return / Annualized Risk (both raw).</t>
+          <t>Weekly R5 portfolio summary from step-04 CNN all_h{k}.xlsx and step-05 benchmark h{k}.xlsx (weekly/). Paper reference: Table I.</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>H-L: eval horizon H1 (signal at t, return over 1st future rebalance period).</t>
+          <t>Return column: Annualized Return (raw portfolio return, annualized). NOT Annualized Active Return.</t>
         </is>
       </c>
     </row>
@@ -536,7 +536,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>DH Ret2 / DH Ret3: H-L (DH) annualized return at eval horizons H2 / H3 (2nd / 3rd future rebalance period).</t>
+          <t>Sharpe column: Sharpe Ratio = Annualized Return / Annualized Risk (both raw).</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Turnover row: monthly turnover on H-L (DH), paper Table I / GKX (2020) convention (R5 one-week holding ≈ 0.25 month; scaled from backtest Turnover (annualized)).</t>
+          <t>H-L: eval horizon H1 (signal at t, return over 1st future rebalance period).</t>
         </is>
       </c>
     </row>
@@ -559,6 +559,30 @@
         </is>
       </c>
       <c r="B12" t="inlineStr">
+        <is>
+          <t>DH Ret2 / DH Ret3: H-L (DH) annualized return at eval horizons H2 / H3 (2nd / 3rd future rebalance period).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Turnover row: monthly turnover on H-L (DH), paper Table I/II / GKX (2020) convention (holding ≈ 0.25 month(s); scaled from backtest Turnover (annualized)).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
         <is>
           <t>H-L and DH Ret2/Ret3 return stars use Newey-West t-stat on the long-short spread.</t>
         </is>

</xml_diff>